<commit_message>
Update import spec for battery
</commit_message>
<xml_diff>
--- a/import-specification/devices/inverter.xlsx
+++ b/import-specification/devices/inverter.xlsx
@@ -203,7 +203,7 @@
     <t>FT_AC_TOTAL</t>
   </si>
   <si>
-    <t>hour</t>
+    <t>h</t>
   </si>
   <si>
     <t>Feed in Time Total AC</t>
@@ -305,7 +305,7 @@
     <t>Grid impedance</t>
   </si>
   <si>
-    <t>R_ISO</t>
+    <t>R_ISO[1..3]</t>
   </si>
   <si>
     <t>kOhm</t>

</xml_diff>